<commit_message>
docs(preuves): reformule les livrables à l'infinitif
Aligner README, en-têtes de scripts et tableur sur la convention du dépôt
(commit 8c7f695) : infinitif, phrases courtes, sans ton explicatif.

Nommer l'objet de chaque script en tête de fichier — démontrer le
correctif — avec la cible, la méthode et les résultats attendus avant et
après, en quelques lignes.

Tableur : colonnes « Abus possible » et « Impact » à la place des
formulations longues, textes resserrés, feuille « Protocole » en dix
entrées.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rqrp45GbJ3567mSYocbzvF
</commit_message>
<xml_diff>
--- a/audit/preuves/failles-et-correctifs.xlsx
+++ b/audit/preuves/failles-et-correctifs.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Failles et preuves" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Mode d'emploi" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="Protocole" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="107">
-  <si>
-    <t>bibble-ai — failles constatées, preuves et correctifs</t>
-  </si>
-  <si>
-    <t>Chaque faille dispose d'un script qui l'exploite réellement. Le même script, rejoué après correction, doit échouer à l'exploiter : c'est la preuve. Les scripts s'exécutent sur une copie locale du site — jamais sur le site en ligne.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="106">
+  <si>
+    <t>bibble-ai — failles, correctifs et preuves d'exécution</t>
+  </si>
+  <si>
+    <t>Démontrer chaque correctif par l'exécution : un script exploite la faille, le même script échoue à l'exploiter une fois le correctif appliqué. Exécution sur copie locale, sans toucher au site en ligne ni aux comptes Stripe et HeyGen.</t>
   </si>
   <si>
     <t>N°</t>
@@ -26,10 +26,10 @@
     <t>Faille</t>
   </si>
   <si>
-    <t>Ce qu'une personne peut en faire</t>
-  </si>
-  <si>
-    <t>Conséquence pour l'entreprise</t>
+    <t>Abus possible</t>
+  </si>
+  <si>
+    <t>Impact</t>
   </si>
   <si>
     <t>Gravité</t>
@@ -47,16 +47,16 @@
     <t>Commande à exécuter</t>
   </si>
   <si>
-    <t>Résultat attendu AVANT correctif</t>
+    <t>Attendu AVANT correctif</t>
   </si>
   <si>
     <t>Preuve AVANT</t>
   </si>
   <si>
-    <t>Correctif prévu</t>
-  </si>
-  <si>
-    <t>Résultat attendu APRÈS correctif</t>
+    <t>Correctif</t>
+  </si>
+  <si>
+    <t>Attendu APRÈS correctif</t>
   </si>
   <si>
     <t>Preuve APRÈS</t>
@@ -65,13 +65,13 @@
     <t>Statut</t>
   </si>
   <si>
-    <t>Un client peut s'attribuer des crédits gratuits</t>
-  </si>
-  <si>
-    <t>Toute personne inscrite peut, depuis la console de son navigateur et en une seule ligne, porter son solde à 9 999 crédits et passer son compte en plan Pro. Aucun outil ni compétence particulière n'est nécessaire : la clé qui le permet est publiée dans le code du site.</t>
-  </si>
-  <si>
-    <t>L'abonnement perd toute valeur : chacun peut générer autant de vidéos qu'il veut sans payer. Chaque vidéo produite est facturée à l'entreprise par HeyGen.</t>
+    <t>Attribution de crédits par l'utilisateur lui-même</t>
+  </si>
+  <si>
+    <t>Porter son solde à 9 999 crédits et passer en plan Pro depuis la console du navigateur, avec la clé publiée dans le code du site.</t>
+  </si>
+  <si>
+    <t>Vidéos illimitées sans paiement. Chaque vidéo produite est facturée par HeyGen.</t>
   </si>
   <si>
     <t>Critique</t>
@@ -89,16 +89,16 @@
     <t>node --env-file=audit/preuves/.env.preuves audit/preuves/scripts/01-rls-escalade-credits.mjs</t>
   </si>
   <si>
-    <t>❌ EXPLOITÉ — le solde passe de 2 à 9 999 crédits et le plan de « starter » à « pro » (code de sortie 1)</t>
-  </si>
-  <si>
-    <t>À exécuter — nécessite la base locale</t>
-  </si>
-  <si>
-    <t>Interdire au client de modifier lui-même les colonnes « crédits » et « plan » : seules les fonctions du serveur pourront y toucher.</t>
-  </si>
-  <si>
-    <t>✅ BLOQUÉ — 0 ligne modifiée, le solde reste à 2 crédits (code de sortie 0)</t>
+    <t>❌ Solde porté à 9 999 crédits, plan « pro » — code 1</t>
+  </si>
+  <si>
+    <t>À exécuter — base locale requise</t>
+  </si>
+  <si>
+    <t>Réserver la modification de « crédits » et « plan » au serveur.</t>
+  </si>
+  <si>
+    <t>✅ Modification refusée, solde inchangé — code 0</t>
   </si>
   <si>
     <t>En attente du correctif</t>
@@ -107,13 +107,13 @@
     <t>À corriger</t>
   </si>
   <si>
-    <t>Un client peut accéder aux vidéos d'un autre client</t>
-  </si>
-  <si>
-    <t>Un compte connecté peut demander le téléchargement ou le statut de la vidéo d'un autre client. Les deux routes concernées n'ont jamais vérifié à qui appartient la vidéo demandée.</t>
-  </si>
-  <si>
-    <t>Fuite de contenus clients : script publicitaire, avatar choisi, message commercial. Confidentialité rompue entre clients, y compris entre concurrents d'un même secteur.</t>
+    <t>Accès aux vidéos d'un autre client</t>
+  </si>
+  <si>
+    <t>Télécharger et suivre la vidéo d'un autre client à partir de son identifiant.</t>
+  </si>
+  <si>
+    <t>Fuite de contenus clients : script publicitaire, avatar, message commercial.</t>
   </si>
   <si>
     <t>Élevée</t>
@@ -131,25 +131,25 @@
     <t>node --env-file=audit/preuves/.env.preuves audit/preuves/scripts/02-idor-videos.mjs</t>
   </si>
   <si>
-    <t>❌ EXPLOITÉ — la demande portant sur la vidéo d'autrui reçoit la même réponse que sur sa propre vidéo : aucun refus (code de sortie 1)</t>
-  </si>
-  <si>
-    <t>À exécuter — nécessite la base locale et l'application lancée</t>
-  </si>
-  <si>
-    <t>Vérifier que la vidéo demandée appartient à la personne connectée, avant tout traitement et avant tout appel au prestataire vidéo.</t>
-  </si>
-  <si>
-    <t>✅ BLOQUÉ — les deux routes répondent « accès refusé » (403) (code de sortie 0)</t>
-  </si>
-  <si>
-    <t>Une notification de paiement rejouée crédite deux fois</t>
-  </si>
-  <si>
-    <t>Stripe renvoie automatiquement une notification lorsqu'il ne reçoit pas de confirmation — ce que l'application provoque elle-même en signalant une erreur. Chaque renvoi réattribue le plein montant de crédits du plan.</t>
-  </si>
-  <si>
-    <t>Des crédits distribués en double, voire en boucle, sans paiement correspondant. L'historique des crédits comporte des lignes fantômes : les comptes ne tombent plus juste.</t>
+    <t>❌ Réponses identiques sur sa vidéo et celle d'autrui — code 1</t>
+  </si>
+  <si>
+    <t>À exécuter — base locale et application requises</t>
+  </si>
+  <si>
+    <t>Vérifier la propriété de la vidéo avant tout traitement.</t>
+  </si>
+  <si>
+    <t>✅ Accès refusé (403) sur la vidéo d'autrui — code 0</t>
+  </si>
+  <si>
+    <t>Notification de paiement rejouée</t>
+  </si>
+  <si>
+    <t>Recevoir deux fois les crédits lorsque Stripe renvoie la notification — renvoi que l'application déclenche elle-même en signalant une erreur.</t>
+  </si>
+  <si>
+    <t>Crédits attribués sans paiement. Historique des crédits faussé.</t>
   </si>
   <si>
     <t>src/app/api/webhooks/stripe/route.ts:46-296</t>
@@ -164,22 +164,22 @@
     <t>node --env-file=audit/preuves/.env.preuves audit/preuves/scripts/03-idempotence-webhook.mjs</t>
   </si>
   <si>
-    <t>❌ EXPLOITÉ — le même événement envoyé deux fois produit 2 attributions de crédits au lieu d'une (code de sortie 1)</t>
-  </si>
-  <si>
-    <t>Enregistrer l'identifiant de chaque notification traitée et ignorer immédiatement toute répétition.</t>
-  </si>
-  <si>
-    <t>✅ BLOQUÉ — une seule attribution malgré le renvoi (code de sortie 0)</t>
-  </si>
-  <si>
-    <t>La date de début d'abonnement enregistrée est fausse</t>
-  </si>
-  <si>
-    <t>Ce n'est pas un abus volontaire mais une erreur de programmation : la date de début d'abonnement reçoit la date de fin. Toutes les périodes enregistrées durent donc zéro jour.</t>
-  </si>
-  <si>
-    <t>Impossible de savoir depuis quand un client est abonné. Tout calcul de renouvellement, de remboursement au prorata ou de relance repose sur une donnée fausse.</t>
+    <t>❌ 2 attributions de crédits pour 1 événement — code 1</t>
+  </si>
+  <si>
+    <t>Mémoriser les notifications traitées, ignorer les répétitions.</t>
+  </si>
+  <si>
+    <t>✅ 1 seule attribution malgré le renvoi — code 0</t>
+  </si>
+  <si>
+    <t>Date de début d'abonnement erronée</t>
+  </si>
+  <si>
+    <t>Aucun abus : erreur de programmation.</t>
+  </si>
+  <si>
+    <t>Périodes d'abonnement de durée nulle. Calculs de renouvellement et de prorata faussés.</t>
   </si>
   <si>
     <t>Moyenne</t>
@@ -197,28 +197,28 @@
     <t>node --env-file=audit/preuves/.env.preuves audit/preuves/scripts/04-periode-abonnement.mjs</t>
   </si>
   <si>
-    <t>❌ EXPLOITÉ — pour une période allant du 01/08 au 01/09, la fonction renvoie 01/09 comme début ET comme fin (code de sortie 1)</t>
-  </si>
-  <si>
-    <t>✔ Exécutée le 2026-08-04 — résultat conforme (aucun prérequis)</t>
-  </si>
-  <si>
-    <t>Utiliser la date de début là où la date de début est attendue.</t>
-  </si>
-  <si>
-    <t>✅ BLOQUÉ — début 01/08 et fin 01/09, deux dates distinctes (code de sortie 0)</t>
-  </si>
-  <si>
-    <t>Une référence tarifaire manquante fausse l'attribution des crédits</t>
-  </si>
-  <si>
-    <t>Les six tarifs sont reliés aux plans par une table de correspondance. Si une référence n'est pas renseignée, son entrée devient vide ; plusieurs références manquantes se remplacent alors les unes les autres et la table se mélange, sans le moindre signal.</t>
-  </si>
-  <si>
-    <t>Constaté à l'exécution : la table tombe à 4 entrées au lieu de 6 et l'entrée vide vaut 15 crédits, le quota du plan Pro. Un abonné Starter peut donc recevoir le quota Pro — ou, à l'inverse, un client payant ne rien recevoir pendant que le paiement est considéré comme traité.</t>
-  </si>
-  <si>
-    <t>src/lib/stripe.ts (PLAN_CREDITS) ; src/app/api/webhooks/stripe/route.ts:20-30</t>
+    <t>❌ Période du 01/08 au 01/09 → début = fin = 01/09 — code 1</t>
+  </si>
+  <si>
+    <t>✔ Exécutée le 2026-08-04 — conforme</t>
+  </si>
+  <si>
+    <t>Renseigner la date de début avec la date de début.</t>
+  </si>
+  <si>
+    <t>✅ Début 01/08, fin 01/09 — code 0</t>
+  </si>
+  <si>
+    <t>Table des tarifs incomplète</t>
+  </si>
+  <si>
+    <t>Aucun abus : défaut de construction déclenché par une référence tarifaire absente.</t>
+  </si>
+  <si>
+    <t>Constaté à l'exécution : 4 entrées au lieu de 6, entrée vide à 15 crédits. Un abonné Starter reçoit le quota Pro ; un tarif inconnu est accepté sans aucun crédit attribué.</t>
+  </si>
+  <si>
+    <t>src/lib/stripe.ts ; src/app/api/webhooks/stripe/route.ts:20-30</t>
   </si>
   <si>
     <t>B3.5</t>
@@ -230,25 +230,22 @@
     <t>node --env-file=audit/preuves/.env.preuves audit/preuves/scripts/05-mapping-price-ids.mjs</t>
   </si>
   <si>
-    <t>❌ EXPLOITÉ — 4 entrées au lieu de 6, l'entrée vide vaut 15 crédits ; un tarif inconnu obtient une réponse « traité » sans qu'aucun crédit ne soit attribué (code de sortie 1)</t>
-  </si>
-  <si>
-    <t>✔ Exécutée le 2026-08-04 — résultat conforme (volet « table de correspondance »)</t>
-  </si>
-  <si>
-    <t>Écarter les références vides à la construction de la table, et signaler bruyamment tout tarif inconnu au lieu de l'ignorer silencieusement.</t>
-  </si>
-  <si>
-    <t>✅ BLOQUÉ — aucune entrée vide dans la table, et un tarif inconnu déclenche une alerte (code de sortie 0)</t>
-  </si>
-  <si>
-    <t>Cinq vidéos peuvent être générées avec un seul crédit</t>
-  </si>
-  <si>
-    <t>En lançant plusieurs générations au même instant, toutes lisent le solde avant que la première ne l'ait diminué. Toutes passent le contrôle et toutes aboutissent. Avec 1 crédit, 5 requêtes simultanées produisent 5 vidéos.</t>
-  </si>
-  <si>
-    <t>Chaque vidéo excédentaire est facturée à l'entreprise par le prestataire sans contrepartie. L'abus ne demande aucune compétence : il suffit de cliquer plusieurs fois.</t>
+    <t>❌ 4 entrées au lieu de 6, clé vide à 15 crédits — code 1</t>
+  </si>
+  <si>
+    <t>Écarter les entrées vides, signaler tout tarif inconnu.</t>
+  </si>
+  <si>
+    <t>✅ Aucune entrée vide, tarif inconnu signalé — code 0</t>
+  </si>
+  <si>
+    <t>Générations simultanées avec un seul crédit</t>
+  </si>
+  <si>
+    <t>Lancer cinq générations au même instant et obtenir cinq vidéos avec un crédit.</t>
+  </si>
+  <si>
+    <t>Vidéos excédentaires facturées sans contrepartie. Aucune compétence requise.</t>
   </si>
   <si>
     <t>src/app/api/generate-video/route.ts:98-181</t>
@@ -263,78 +260,76 @@
     <t>node --env-file=audit/preuves/.env.preuves audit/preuves/scripts/06-course-credits.mjs</t>
   </si>
   <si>
-    <t>❌ EXPLOITÉ — 5 vidéos lancées, 1 seul crédit débité, 4 vidéos offertes (code de sortie 1)</t>
-  </si>
-  <si>
-    <t>Débiter le crédit en une opération unique et indivisible en base, avant l'appel au prestataire, et le rembourser si la génération échoue.</t>
-  </si>
-  <si>
-    <t>✅ BLOQUÉ — 1 vidéo lancée, les 4 autres requêtes refusées (code de sortie 0)</t>
-  </si>
-  <si>
-    <t>Comment rejouer les preuves</t>
+    <t>❌ 5 vidéos lancées, 1 crédit débité — code 1</t>
+  </si>
+  <si>
+    <t>Débiter le crédit en une opération indivisible avant l'appel au prestataire, rembourser en cas d'échec.</t>
+  </si>
+  <si>
+    <t>✅ 1 vidéo lancée, 4 requêtes refusées — code 0</t>
+  </si>
+  <si>
+    <t>Protocole</t>
   </si>
   <si>
     <t>Principe</t>
   </si>
   <si>
-    <t>Chaque faille est exploitée pour de bon par un script. Le script se termine par « ❌ EXPLOITÉ » tant que la faille est présente, et par « ✅ BLOQUÉ » une fois le correctif appliqué. La preuve tient dans ce basculement, obtenu avec exactement la même commande.</t>
-  </si>
-  <si>
-    <t>Où cela s'exécute</t>
-  </si>
-  <si>
-    <t>Sur une copie du site installée sur un poste de travail, avec une base de données vierge créée à partir des fichiers du projet. Ni le site en ligne, ni la base réelle, ni le compte Stripe ne sont sollicités : un garde-fou dans les scripts refuse toute cible autre que locale.</t>
-  </si>
-  <si>
-    <t>Aucun compte tiers requis</t>
-  </si>
-  <si>
-    <t>Les notifications de paiement sont fabriquées et signées localement. Aucune vidéo n'est commandée au prestataire, donc aucune facturation n'est déclenchée par les tests.</t>
+    <t>Exploiter la faille avant correctif, échouer à l'exploiter après. Même commande, deux résultats.</t>
+  </si>
+  <si>
+    <t>Portée</t>
+  </si>
+  <si>
+    <t>Base locale créée depuis les fichiers du projet. Ni le site en ligne, ni la base réelle, ni le compte Stripe ne sont sollicités.</t>
+  </si>
+  <si>
+    <t>Comptes tiers</t>
+  </si>
+  <si>
+    <t>Aucun. Notifications de paiement signées localement, aucune vidéo commandée au prestataire.</t>
   </si>
   <si>
     <t>1. Préparer</t>
   </si>
   <si>
-    <t>npx supabase init puis npx supabase start — installe une base locale à partir des fichiers du projet. Copier audit/preuves/.env.preuves.example en .env.preuves et y coller les deux clés affichées.</t>
-  </si>
-  <si>
-    <t>2. Lancer le site en local</t>
+    <t>npx supabase init puis npx supabase start. Copier .env.preuves.example en .env.preuves, y coller les deux clés affichées.</t>
+  </si>
+  <si>
+    <t>2. Lancer l'application</t>
   </si>
   <si>
     <t>npm run dev, dans un second terminal.</t>
   </si>
   <si>
-    <t>3. Capturer l'état AVANT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">node --env-file=audit/preuves/.env.preuves audit/preuves/scripts/run-all.mjs avant
-Les six scripts s'exécutent et leurs sorties horodatées sont archivées dans audit/preuves/resultats/avant/, avec un récapitulatif.</t>
+    <t>3. Capturer l'avant</t>
+  </si>
+  <si>
+    <t>run-all.mjs avant — sorties horodatées archivées dans resultats/avant/.</t>
   </si>
   <si>
     <t>4. Figer le point de départ</t>
   </si>
   <si>
-    <t>git tag preuve-avant — repère posé sur la version non corrigée, pour que la démonstration reste rejouable même après les correctifs.</t>
+    <t>git tag preuve-avant — conserver la version non corrigée, rejouable.</t>
   </si>
   <si>
     <t>5. Corriger</t>
   </si>
   <si>
-    <t>Les correctifs sont appliqués dans l'ordre du plan : d'abord les crédits gratuits, puis les crédits multiples, puis l'accès aux vidéos, puis les notifications de paiement.</t>
-  </si>
-  <si>
-    <t>6. Capturer l'état APRÈS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">node --env-file=audit/preuves/.env.preuves audit/preuves/scripts/run-all.mjs apres
-Les six lignes doivent être passées de ❌ à ✅. C'est le livrable de recette.</t>
-  </si>
-  <si>
-    <t>Lecture des résultats</t>
-  </si>
-  <si>
-    <t>Code 0 = ✅ la faille n'est plus exploitable. Code 1 = ❌ la faille est exploitable. Code 2 = ⚠️ le test n'a pas pu conclure (un prérequis manquait).</t>
+    <t>Appliquer les correctifs dans l'ordre du plan.</t>
+  </si>
+  <si>
+    <t>6. Capturer l'après</t>
+  </si>
+  <si>
+    <t>run-all.mjs apres — les six lignes doivent passer de ❌ à ✅.</t>
+  </si>
+  <si>
+    <t>Codes</t>
+  </si>
+  <si>
+    <t>0 = ✅ faille non exploitable. 1 = ❌ faille exploitable. 2 = ⚠️ prérequis manquant.</t>
   </si>
 </sst>
 </file>
@@ -893,17 +888,18 @@
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="52" customWidth="1"/>
-    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="46" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
     <col min="8" max="8" width="28" customWidth="1"/>
-    <col min="9" max="10" width="46" customWidth="1"/>
-    <col min="11" max="11" width="34" customWidth="1"/>
-    <col min="12" max="12" width="46" customWidth="1"/>
-    <col min="13" max="13" width="42" customWidth="1"/>
-    <col min="14" max="14" width="26" customWidth="1"/>
+    <col min="9" max="9" width="46" customWidth="1"/>
+    <col min="10" max="10" width="42" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
+    <col min="12" max="12" width="44" customWidth="1"/>
+    <col min="13" max="13" width="40" customWidth="1"/>
+    <col min="14" max="14" width="24" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
   </cols>
   <sheetData>
@@ -992,7 +988,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" ht="108" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="78" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>1</v>
       </c>
@@ -1039,7 +1035,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" ht="108" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="78" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="13">
         <v>2</v>
       </c>
@@ -1086,7 +1082,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" ht="108" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" ht="78" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>3</v>
       </c>
@@ -1133,7 +1129,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" ht="108" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="78" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="13">
         <v>4</v>
       </c>
@@ -1180,7 +1176,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" ht="108" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="78" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>5</v>
       </c>
@@ -1212,13 +1208,13 @@
         <v>72</v>
       </c>
       <c r="K8" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="L8" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="L8" s="6" t="s">
+      <c r="M8" s="11" t="s">
         <v>74</v>
-      </c>
-      <c r="M8" s="11" t="s">
-        <v>75</v>
       </c>
       <c r="N8" s="6" t="s">
         <v>29</v>
@@ -1227,45 +1223,45 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" ht="108" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="78" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="13">
         <v>6</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="D9" s="15" t="s">
         <v>77</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>78</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F9" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="H9" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="H9" s="17" t="s">
+      <c r="I9" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="I9" s="17" t="s">
+      <c r="J9" s="18" t="s">
         <v>82</v>
-      </c>
-      <c r="J9" s="18" t="s">
-        <v>83</v>
       </c>
       <c r="K9" s="19" t="s">
         <v>26</v>
       </c>
       <c r="L9" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="M9" s="20" t="s">
         <v>84</v>
-      </c>
-      <c r="M9" s="20" t="s">
-        <v>85</v>
       </c>
       <c r="N9" s="15" t="s">
         <v>29</v>
@@ -1297,89 +1293,89 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" ht="58" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="26" t="s">
+    </row>
+    <row r="4" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="27" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="4" ht="58" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="27" t="s">
+      <c r="C4" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="28" t="s">
+    </row>
+    <row r="5" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="25" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="5" ht="58" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="25" t="s">
+      <c r="C5" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="C5" s="26" t="s">
+    </row>
+    <row r="6" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="27" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="6" ht="58" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
+      <c r="C6" s="28" t="s">
         <v>93</v>
       </c>
-      <c r="C6" s="28" t="s">
+    </row>
+    <row r="7" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="25" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="7" ht="58" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="25" t="s">
+      <c r="C7" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="C7" s="26" t="s">
+    </row>
+    <row r="8" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="27" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="8" ht="58" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="27" t="s">
+      <c r="C8" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="C8" s="28" t="s">
+    </row>
+    <row r="9" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="25" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="9" ht="58" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="25" t="s">
+      <c r="C9" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="C9" s="26" t="s">
+    </row>
+    <row r="10" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B10" s="27" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="10" ht="58" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="27" t="s">
+      <c r="C10" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="C10" s="28" t="s">
+    </row>
+    <row r="11" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B11" s="25" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="11" ht="58" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="25" t="s">
+      <c r="C11" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="26" t="s">
+    </row>
+    <row r="12" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="27" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="12" ht="58" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="27" t="s">
+      <c r="C12" s="28" t="s">
         <v>105</v>
-      </c>
-      <c r="C12" s="28" t="s">
-        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>